<commit_message>
Auto: refresh raw URLs for phxnkhlay
</commit_message>
<xml_diff>
--- a/data/phxnkhlay_all_raw.xlsx
+++ b/data/phxnkhlay_all_raw.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,16 +446,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>markpom</t>
+          <t>alturl_bulk_shorten.py</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>.github/workflows/main.yml</t>
+          <t>.github/workflows/shorten-urls.yml</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>937</v>
+        <v>1834</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -464,23 +464,23 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/.github/workflows/main.yml</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/alturl_bulk_shorten.py/main/.github/workflows/shorten-urls.yml</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>markpom</t>
+          <t>alturl_bulk_shorten.py</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MP01JANUARI2027</t>
+          <t>alturl_bulk_shorten.py</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>588660</v>
+        <v>13580</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -489,23 +489,23 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP01JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/alturl_bulk_shorten.py/main/alturl_bulk_shorten.py</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>markpom</t>
+          <t>alturl_bulk_shorten.py</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MP02JANUARI2027</t>
+          <t>hasil_shorturl.csv</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>588660</v>
+        <v>3878</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP02JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/alturl_bulk_shorten.py/main/hasil_shorturl.csv</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MP03JANUARI2027</t>
+          <t>.github/workflows/main.yml</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>588660</v>
+        <v>937</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP03JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/.github/workflows/main.yml</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MP04JANUARI2027</t>
+          <t>MP01JANUARI2027</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP04JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP01JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MP05JANUARI2027</t>
+          <t>MP02JANUARI2027</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP05JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP02JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MP06JANUARI2027</t>
+          <t>MP03JANUARI2027</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP06JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP03JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MP07JANUARI2027</t>
+          <t>MP04JANUARI2027</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -639,7 +639,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP07JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP04JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MP08JANUARI2027</t>
+          <t>MP05JANUARI2027</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP08JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP05JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MP09JANUARI2027</t>
+          <t>MP06JANUARI2027</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -689,7 +689,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP09JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP06JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MP10JANUARI2027</t>
+          <t>MP07JANUARI2027</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP10JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP07JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MP11JANUARI2027</t>
+          <t>MP08JANUARI2027</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -739,7 +739,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP11JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP08JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MP12JANUARI2027</t>
+          <t>MP09JANUARI2027</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP12JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP09JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MP13JANUARI2027</t>
+          <t>MP10JANUARI2027</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP13JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP10JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MP14JANUARI2027</t>
+          <t>MP11JANUARI2027</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -814,7 +814,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP14JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP11JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MP15JANUARI2027</t>
+          <t>MP12JANUARI2027</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP15JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP12JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MP16JANUARI2027</t>
+          <t>MP13JANUARI2027</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP16JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP13JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MP17JANUARI2027</t>
+          <t>MP14JANUARI2027</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -889,7 +889,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP17JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP14JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MP18JANUARI2027</t>
+          <t>MP15JANUARI2027</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP18JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP15JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MP19JANUARI2027</t>
+          <t>MP16JANUARI2027</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -939,7 +939,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP19JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP16JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MP20JANUARI2027</t>
+          <t>MP17JANUARI2027</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP20JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP17JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MP21JANUARI2027</t>
+          <t>MP18JANUARI2027</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -989,7 +989,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP21JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP18JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MP22JANUARI2027</t>
+          <t>MP19JANUARI2027</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP22JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP19JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MP23JANUARI2027</t>
+          <t>MP20JANUARI2027</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP23JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP20JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MP24JANUARI2027</t>
+          <t>MP21JANUARI2027</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP24JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP21JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MP25JANUARI2027</t>
+          <t>MP22JANUARI2027</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP25JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP22JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MP26JANUARI2027</t>
+          <t>MP23JANUARI2027</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP26JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP23JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MP27JANUARI2027</t>
+          <t>MP24JANUARI2027</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP27JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP24JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MP28JANUARI2027</t>
+          <t>MP25JANUARI2027</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP28JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP25JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MP29JANUARI2027</t>
+          <t>MP26JANUARI2027</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP29JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP26JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MP30JANUARI2027</t>
+          <t>MP27JANUARI2027</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP30JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP27JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MP31JANUARI2027</t>
+          <t>MP28JANUARI2027</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP31JANUARI2027</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP28JANUARI2027</t>
         </is>
       </c>
     </row>
@@ -1251,11 +1251,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>update_github_file.py</t>
+          <t>MP29JANUARI2027</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>14662</v>
+        <v>588660</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1264,23 +1264,23 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/update_github_file.py</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP29JANUARI2027</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>URL-GENERATOR</t>
+          <t>markpom</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>.github/workflows/raw-urls.yml</t>
+          <t>MP30JANUARI2027</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2168</v>
+        <v>588660</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1289,23 +1289,23 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/.github/workflows/raw-urls.yml</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP30JANUARI2027</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>URL-GENERATOR</t>
+          <t>markpom</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>data/uppermoon77_all_raw.csv</t>
+          <t>MP31JANUARI2027</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>42049</v>
+        <v>588660</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1314,23 +1314,23 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/data/uppermoon77_all_raw.csv</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/MP31JANUARI2027</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>URL-GENERATOR</t>
+          <t>markpom</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>data/uppermoon77_all_raw.xlsx</t>
+          <t>update_github_file.py</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>15157</v>
+        <v>14662</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/data/uppermoon77_all_raw.xlsx</t>
+          <t>https://raw.githubusercontent.com/phxnkhlay/markpom/main/update_github_file.py</t>
         </is>
       </c>
     </row>
@@ -1351,18 +1351,143 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>.github/workflows/raw-urls.yml</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2168</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/.github/workflows/raw-urls.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>URL-GENERATOR</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>data/phxnkhlay_all_raw.csv</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>4252</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/data/phxnkhlay_all_raw.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>URL-GENERATOR</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>data/phxnkhlay_all_raw.xlsx</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6059</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/data/phxnkhlay_all_raw.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>URL-GENERATOR</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>data/uppermoon77_all_raw.csv</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>42049</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/data/uppermoon77_all_raw.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>URL-GENERATOR</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>data/uppermoon77_all_raw.xlsx</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>15157</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/data/uppermoon77_all_raw.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>URL-GENERATOR</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>generate_all_repos_raw_urls.py</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C43" t="n">
         <v>6525</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/phxnkhlay/URL-GENERATOR/main/generate_all_repos_raw_urls.py</t>
         </is>

</xml_diff>